<commit_message>
preenchimento da tabela de dicionario de dados
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="109">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -114,10 +114,43 @@
     <t xml:space="preserve">matrícula</t>
   </si>
   <si>
+    <t xml:space="preserve">Campo da Matrícula do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e-mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEXt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de E-mail do funcionário</t>
+  </si>
+  <si>
     <t xml:space="preserve">cliente</t>
   </si>
   <si>
+    <t xml:space="preserve">Chave Primária de identificação do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do Nome do cliente</t>
+  </si>
+  <si>
     <t xml:space="preserve">equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do Nome do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação da situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do Nome da situação</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -794,7 +827,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -959,596 +992,641 @@
       <c r="G13" s="12"/>
       <c r="H13" s="11"/>
       <c r="I13" s="14" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="12"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C15" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9" t="s">
+      <c r="D15" s="9"/>
+      <c r="E15" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G15" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H14" s="7"/>
-      <c r="I14" s="10" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="11" t="s">
+      <c r="H15" s="7"/>
+      <c r="I15" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C16" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13" t="s">
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G15" s="12"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16" s="7" t="s">
+      <c r="G16" s="12"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C17" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9" t="s">
+      <c r="D17" s="9"/>
+      <c r="E17" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F17" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G17" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H16" s="7"/>
-      <c r="I16" s="10" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B17" s="11" t="s">
+      <c r="H17" s="7"/>
+      <c r="I17" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C18" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13" t="s">
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G17" s="12"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="10"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="14" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="14"/>
+      <c r="A19" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="7"/>
+      <c r="I19" s="10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="10"/>
+      <c r="A20" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="12"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="14" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="14"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="10"/>
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="14"/>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="14"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="10"/>
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="14"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="14"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="10"/>
+      <c r="A26" s="11"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="14"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="10"/>
+      <c r="A28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="14"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="14"/>
+      <c r="A29" s="7"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7"/>
-      <c r="B30" s="7"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="10"/>
+      <c r="A30" s="11"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="14"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="14"/>
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="10"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7"/>
-      <c r="B32" s="7"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="10"/>
+      <c r="A32" s="11"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="14"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="14"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="10"/>
+      <c r="A34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="13"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="14"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="14"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="10"/>
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="14"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="14"/>
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="10"/>
+      <c r="A38" s="11"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="14"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="14"/>
+      <c r="A39" s="7"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7"/>
-      <c r="B40" s="7"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="10"/>
+      <c r="A40" s="11"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="14"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="14"/>
+      <c r="A41" s="7"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="8"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7"/>
-      <c r="B42" s="7"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="7"/>
-      <c r="I42" s="10"/>
+      <c r="A42" s="11"/>
+      <c r="B42" s="11"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="11"/>
+      <c r="I42" s="14"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="12"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="14"/>
+      <c r="A43" s="7"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="7"/>
-      <c r="I44" s="10"/>
+      <c r="A44" s="11"/>
+      <c r="B44" s="11"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="11"/>
+      <c r="I44" s="14"/>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="11"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="12"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="14"/>
+      <c r="A45" s="7"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="8"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="10"/>
+      <c r="A46" s="11"/>
+      <c r="B46" s="11"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="14"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="11"/>
-      <c r="B47" s="11"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="11"/>
-      <c r="I47" s="14"/>
+      <c r="A47" s="7"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7"/>
-      <c r="B48" s="7"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="9"/>
-      <c r="G48" s="8"/>
-      <c r="H48" s="7"/>
-      <c r="I48" s="10"/>
+      <c r="A48" s="11"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="13"/>
+      <c r="F48" s="13"/>
+      <c r="G48" s="12"/>
+      <c r="H48" s="11"/>
+      <c r="I48" s="14"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="11"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="12"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="14"/>
+      <c r="A49" s="7"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7"/>
-      <c r="B50" s="7"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="9"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="7"/>
-      <c r="I50" s="10"/>
+      <c r="A50" s="11"/>
+      <c r="B50" s="11"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="12"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="14"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="11"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="12"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="12"/>
-      <c r="H51" s="11"/>
-      <c r="I51" s="14"/>
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+      <c r="G51" s="8"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7"/>
-      <c r="B52" s="7"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9"/>
-      <c r="G52" s="8"/>
-      <c r="H52" s="7"/>
-      <c r="I52" s="10"/>
+      <c r="A52" s="11"/>
+      <c r="B52" s="11"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="13"/>
+      <c r="E52" s="13"/>
+      <c r="F52" s="13"/>
+      <c r="G52" s="12"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="14"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="11"/>
-      <c r="B53" s="11"/>
-      <c r="C53" s="12"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
-      <c r="F53" s="13"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="11"/>
-      <c r="I53" s="14"/>
+      <c r="A53" s="7"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="9"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="7"/>
-      <c r="I54" s="10"/>
+      <c r="A54" s="11"/>
+      <c r="B54" s="11"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="13"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="12"/>
+      <c r="H54" s="11"/>
+      <c r="I54" s="14"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="11"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="12"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="14"/>
+      <c r="A55" s="7"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="8"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7"/>
-      <c r="B56" s="7"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="9"/>
-      <c r="G56" s="8"/>
-      <c r="H56" s="7"/>
-      <c r="I56" s="10"/>
+      <c r="A56" s="11"/>
+      <c r="B56" s="11"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="13"/>
+      <c r="E56" s="13"/>
+      <c r="F56" s="13"/>
+      <c r="G56" s="12"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="14"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="11"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="12"/>
-      <c r="H57" s="11"/>
-      <c r="I57" s="14"/>
+      <c r="A57" s="7"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
+      <c r="F57" s="9"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7"/>
-      <c r="B58" s="7"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9"/>
-      <c r="G58" s="8"/>
-      <c r="H58" s="7"/>
-      <c r="I58" s="10"/>
+      <c r="A58" s="11"/>
+      <c r="B58" s="11"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="13"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="12"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="14"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="11"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="13"/>
-      <c r="E59" s="13"/>
-      <c r="F59" s="13"/>
-      <c r="G59" s="12"/>
-      <c r="H59" s="11"/>
-      <c r="I59" s="14"/>
+      <c r="A59" s="7"/>
+      <c r="B59" s="7"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="7"/>
-      <c r="B60" s="7"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="8"/>
-      <c r="H60" s="7"/>
-      <c r="I60" s="10"/>
+      <c r="A60" s="11"/>
+      <c r="B60" s="11"/>
+      <c r="C60" s="12"/>
+      <c r="D60" s="13"/>
+      <c r="E60" s="13"/>
+      <c r="F60" s="13"/>
+      <c r="G60" s="12"/>
+      <c r="H60" s="11"/>
+      <c r="I60" s="14"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="11"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="12"/>
-      <c r="D61" s="13"/>
-      <c r="E61" s="13"/>
-      <c r="F61" s="13"/>
-      <c r="G61" s="12"/>
-      <c r="H61" s="11"/>
-      <c r="I61" s="14"/>
+      <c r="A61" s="7"/>
+      <c r="B61" s="7"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="9"/>
+      <c r="G61" s="8"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="10"/>
+    </row>
+    <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="11"/>
+      <c r="B62" s="11"/>
+      <c r="C62" s="12"/>
+      <c r="D62" s="13"/>
+      <c r="E62" s="13"/>
+      <c r="F62" s="13"/>
+      <c r="G62" s="12"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="14"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C61" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C62" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E61" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E62" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F61" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F62" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1583,89 +1661,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1673,7 +1751,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>10</v>
@@ -1688,10 +1766,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>16</v>
@@ -1699,16 +1777,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>20</v>
@@ -1717,160 +1795,160 @@
         <v>21</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>20</v>
@@ -1879,65 +1957,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1967,15 +2045,15 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>21</v>
@@ -1983,23 +2061,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2009,27 +2087,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modelo conceitual parcial 8 entidades
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="157">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -78,81 +78,237 @@
     <t xml:space="preserve">funcionários</t>
   </si>
   <si>
+    <t xml:space="preserve">id_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOINCREMENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEXT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do Nome do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIQUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação da função</t>
+  </si>
+  <si>
+    <t xml:space="preserve">status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de identificação do status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_admissao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da data de admissão do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">função</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da Função do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matrícula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da Matrícula do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e-mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de E-mail do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do CPF do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">telefone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de telefone do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">senha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de senha do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação da função</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do nome da função</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cliente</t>
+  </si>
+  <si>
     <t xml:space="preserve">id </t>
   </si>
   <si>
-    <t xml:space="preserve">INT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NÃO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOINCREMENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Primária de identificação do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEXT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do Nome do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">função</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo da Função do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matrícula</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo da Matrícula do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">e-mail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEXt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo de E-mail do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cliente</t>
-  </si>
-  <si>
     <t xml:space="preserve">Chave Primária de identificação do cliente</t>
   </si>
   <si>
+    <t xml:space="preserve">nome_cliente</t>
+  </si>
+  <si>
     <t xml:space="preserve">Campo do Nome do cliente</t>
   </si>
   <si>
+    <t xml:space="preserve">Campo de telefone do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECK(1,3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação da situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de E-mail do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">endereco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de endereço do cliente</t>
+  </si>
+  <si>
     <t xml:space="preserve">equipamento</t>
   </si>
   <si>
     <t xml:space="preserve">Chave Primária de identificação do equipamento</t>
   </si>
   <si>
+    <t xml:space="preserve">nome_equipamento</t>
+  </si>
+  <si>
     <t xml:space="preserve">Campo do Nome do equipamento</t>
   </si>
   <si>
+    <t xml:space="preserve">id_marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARCA / ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação da marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MODELO / ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação do modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIPO / ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação do tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_emissão</t>
+  </si>
+  <si>
     <t xml:space="preserve">situação</t>
   </si>
   <si>
+    <t xml:space="preserve">id_situação </t>
+  </si>
+  <si>
     <t xml:space="preserve">Chave Primária de identificação da situação</t>
   </si>
   <si>
+    <t xml:space="preserve">nome_situação</t>
+  </si>
+  <si>
     <t xml:space="preserve">Campo do Nome da situação</t>
   </si>
   <si>
+    <t xml:space="preserve">marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_funcionario_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_tipo</t>
+  </si>
+  <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
   </si>
   <si>
@@ -258,27 +414,18 @@
     <t xml:space="preserve">Nome civil completo do aluno.</t>
   </si>
   <si>
-    <t xml:space="preserve">cpf</t>
-  </si>
-  <si>
     <t xml:space="preserve">Apenas números. Deve ser único (UNIQUE).</t>
   </si>
   <si>
     <t xml:space="preserve">data_nascimento</t>
   </si>
   <si>
-    <t xml:space="preserve">DATE</t>
-  </si>
-  <si>
     <t xml:space="preserve">Data de nascimento para cálculo de idade.</t>
   </si>
   <si>
     <t xml:space="preserve">email</t>
   </si>
   <si>
-    <t xml:space="preserve">SIM</t>
-  </si>
-  <si>
     <t xml:space="preserve">NULL</t>
   </si>
   <si>
@@ -286,9 +433,6 @@
   </si>
   <si>
     <t xml:space="preserve">id_turma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FK</t>
   </si>
   <si>
     <t xml:space="preserve">tb_turmas(id_turma)</t>
@@ -433,7 +577,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -444,6 +588,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1E3A8A"/>
         <bgColor rgb="FF003366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -502,7 +652,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -535,19 +685,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -557,6 +707,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -827,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -927,8 +1081,8 @@
       <c r="G10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="7"/>
-      <c r="I10" s="10" t="s">
+      <c r="H10" s="10"/>
+      <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
@@ -936,7 +1090,7 @@
       <c r="A11" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="7" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="12" t="s">
@@ -948,8 +1102,8 @@
         <v>21</v>
       </c>
       <c r="G11" s="12"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="14" t="s">
+      <c r="H11" s="14"/>
+      <c r="I11" s="15" t="s">
         <v>26</v>
       </c>
     </row>
@@ -957,53 +1111,61 @@
       <c r="A12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
+      <c r="E12" s="13" t="s">
+        <v>28</v>
+      </c>
       <c r="F12" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="12"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="14" t="s">
-        <v>28</v>
+      <c r="G12" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>29</v>
+      <c r="B13" s="7" t="s">
+        <v>31</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G13" s="12"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="14" t="s">
-        <v>30</v>
+      <c r="G13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="14"/>
+      <c r="I13" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>31</v>
+      <c r="B14" s="7" t="s">
+        <v>33</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
@@ -1011,42 +1173,38 @@
         <v>21</v>
       </c>
       <c r="G14" s="12"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="14" t="s">
-        <v>33</v>
+      <c r="H14" s="14"/>
+      <c r="I14" s="11" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="10" t="s">
-        <v>35</v>
+      <c r="A15" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="12"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="15" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>24</v>
+      <c r="A16" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>38</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>25</v>
@@ -1056,43 +1214,41 @@
       <c r="F16" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G16" s="12"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="14" t="s">
-        <v>36</v>
+      <c r="G16" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" s="14"/>
+      <c r="I16" s="15" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H17" s="7"/>
-      <c r="I17" s="10" t="s">
-        <v>38</v>
+      <c r="A17" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G17" s="12"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="15" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>24</v>
+      <c r="A18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>25</v>
@@ -1102,43 +1258,41 @@
       <c r="F18" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G18" s="12"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="14" t="s">
-        <v>39</v>
+      <c r="G18" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H18" s="14"/>
+      <c r="I18" s="15" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H19" s="7"/>
-      <c r="I19" s="10" t="s">
+      <c r="A19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13" t="s">
         <v>41</v>
       </c>
+      <c r="G19" s="12"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="11" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>24</v>
+      <c r="A20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>47</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>25</v>
@@ -1149,484 +1303,1322 @@
         <v>21</v>
       </c>
       <c r="G20" s="12"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="14" t="s">
-        <v>42</v>
+      <c r="H20" s="14"/>
+      <c r="I20" s="11" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="10"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
+      <c r="A22" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="14"/>
+      <c r="E22" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="14"/>
+      <c r="I22" s="11" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="10"/>
+      <c r="A23" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H23" s="14"/>
+      <c r="I23" s="11" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="12"/>
+      <c r="A24" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="14"/>
+      <c r="F24" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="11" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="10"/>
+      <c r="A25" s="10"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11"/>
-      <c r="B26" s="11"/>
+      <c r="A26" s="10"/>
+      <c r="B26" s="14"/>
       <c r="C26" s="12"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
       <c r="G26" s="12"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="8"/>
+      <c r="A27" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="10"/>
+      <c r="E27" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="10"/>
+      <c r="I27" s="11" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="12"/>
+      <c r="A28" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
+      <c r="F28" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G28" s="12"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="15" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="10"/>
+      <c r="A29" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="12"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
+      <c r="A30" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>59</v>
+      </c>
       <c r="C30" s="12"/>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
       <c r="G30" s="12"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="10"/>
+      <c r="A31" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G31" s="12"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="12"/>
+      <c r="A32" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
+      <c r="E32" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G32" s="12"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="14"/>
+      <c r="H32" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="10"/>
+      <c r="A33" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="12"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="11" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="12"/>
+      <c r="A34" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="14"/>
+      <c r="F34" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G34" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H34" s="14"/>
+      <c r="I34" s="15" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="10"/>
+      <c r="A35" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G35" s="12"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="15" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="12"/>
+      <c r="A36" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
+      <c r="F36" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G36" s="12"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="15" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="10"/>
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
       <c r="C38" s="12"/>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
       <c r="F38" s="13"/>
       <c r="G38" s="12"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="14"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7"/>
-      <c r="B39" s="7"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="10"/>
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="14"/>
+      <c r="I39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="14"/>
+      <c r="A40" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H40" s="10"/>
+      <c r="I40" s="11" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="7"/>
-      <c r="I41" s="10"/>
+      <c r="A41" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" s="12"/>
+      <c r="H41" s="14"/>
+      <c r="I41" s="15" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="12"/>
+      <c r="A42" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
+      <c r="E42" s="13" t="s">
+        <v>28</v>
+      </c>
       <c r="F42" s="13"/>
       <c r="G42" s="12"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="14"/>
+      <c r="H42" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="I42" s="11" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="7"/>
-      <c r="I43" s="10"/>
+      <c r="A43" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F43" s="13"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="I43" s="11" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="12"/>
+      <c r="A44" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
+      <c r="E44" s="13" t="s">
+        <v>28</v>
+      </c>
       <c r="F44" s="13"/>
       <c r="G44" s="12"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="14"/>
+      <c r="H44" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I44" s="11" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="7"/>
-      <c r="I45" s="10"/>
+      <c r="A45" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="13"/>
+      <c r="E45" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F45" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G45" s="12"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="11"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="11"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="12"/>
+      <c r="A46" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="12"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="14"/>
+      <c r="F46" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G46" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="14"/>
+      <c r="I46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7"/>
-      <c r="B47" s="7"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="10"/>
+      <c r="A47" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D47" s="13"/>
+      <c r="E47" s="13"/>
+      <c r="F47" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G47" s="12"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="11"/>
-      <c r="B48" s="11"/>
+      <c r="A48" s="14"/>
+      <c r="B48" s="14"/>
       <c r="C48" s="12"/>
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
       <c r="F48" s="13"/>
       <c r="G48" s="12"/>
-      <c r="H48" s="11"/>
-      <c r="I48" s="14"/>
+      <c r="H48" s="14"/>
+      <c r="I48" s="15"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7"/>
-      <c r="B49" s="7"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="9"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="7"/>
-      <c r="I49" s="10"/>
+      <c r="A49" s="14"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="12"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="12"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="15"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="11"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="13"/>
-      <c r="G50" s="12"/>
-      <c r="H50" s="11"/>
-      <c r="I50" s="14"/>
+      <c r="A50" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G50" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H50" s="10"/>
+      <c r="I50" s="11" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7"/>
-      <c r="B51" s="7"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="9"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="7"/>
-      <c r="I51" s="10"/>
+      <c r="A51" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D51" s="13"/>
+      <c r="E51" s="13"/>
+      <c r="F51" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G51" s="12"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="15" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="11"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="12"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="12"/>
-      <c r="H52" s="11"/>
-      <c r="I52" s="14"/>
+      <c r="A52" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="8"/>
+      <c r="H52" s="10"/>
+      <c r="I52" s="11"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="9"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="7"/>
-      <c r="I53" s="10"/>
+      <c r="A53" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
+      <c r="F53" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G53" s="12"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="15"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="11"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="12"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="12"/>
-      <c r="H54" s="11"/>
-      <c r="I54" s="14"/>
+      <c r="A54" s="10"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="10"/>
+      <c r="I54" s="11"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7"/>
-      <c r="B55" s="7"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="9"/>
-      <c r="F55" s="9"/>
-      <c r="G55" s="8"/>
-      <c r="H55" s="7"/>
-      <c r="I55" s="10"/>
+      <c r="A55" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D55" s="13"/>
+      <c r="E55" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F55" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H55" s="14"/>
+      <c r="I55" s="11" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="11"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="12"/>
+      <c r="A56" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="D56" s="13"/>
       <c r="E56" s="13"/>
-      <c r="F56" s="13"/>
-      <c r="G56" s="12"/>
-      <c r="H56" s="11"/>
-      <c r="I56" s="14"/>
+      <c r="F56" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G56" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H56" s="14"/>
+      <c r="I56" s="11" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7"/>
-      <c r="B57" s="7"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="9"/>
-      <c r="G57" s="8"/>
-      <c r="H57" s="7"/>
-      <c r="I57" s="10"/>
+      <c r="A57" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D57" s="13"/>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G57" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="14"/>
+      <c r="I57" s="11" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="11"/>
-      <c r="B58" s="11"/>
+      <c r="A58" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="C58" s="12"/>
       <c r="D58" s="13"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="13"/>
+      <c r="E58" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F58" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G58" s="12"/>
-      <c r="H58" s="11"/>
-      <c r="I58" s="14"/>
+      <c r="H58" s="14"/>
+      <c r="I58" s="11" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="7"/>
-      <c r="B59" s="7"/>
+      <c r="A59" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
+      <c r="E59" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>21</v>
+      </c>
       <c r="G59" s="8"/>
-      <c r="H59" s="7"/>
-      <c r="I59" s="10"/>
+      <c r="H59" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="I59" s="11" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="11"/>
-      <c r="B60" s="11"/>
+      <c r="A60" s="14"/>
+      <c r="B60" s="14"/>
       <c r="C60" s="12"/>
       <c r="D60" s="13"/>
       <c r="E60" s="13"/>
       <c r="F60" s="13"/>
       <c r="G60" s="12"/>
-      <c r="H60" s="11"/>
-      <c r="I60" s="14"/>
+      <c r="H60" s="14"/>
+      <c r="I60" s="15"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="7"/>
-      <c r="B61" s="7"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="9"/>
-      <c r="G61" s="8"/>
-      <c r="H61" s="7"/>
-      <c r="I61" s="10"/>
+      <c r="A61" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D61" s="13"/>
+      <c r="E61" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F61" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G61" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H61" s="14"/>
+      <c r="I61" s="11" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="11"/>
-      <c r="B62" s="11"/>
-      <c r="C62" s="12"/>
+      <c r="A62" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C62" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="D62" s="13"/>
       <c r="E62" s="13"/>
-      <c r="F62" s="13"/>
-      <c r="G62" s="12"/>
-      <c r="H62" s="11"/>
-      <c r="I62" s="14"/>
-    </row>
+      <c r="F62" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G62" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H62" s="14"/>
+      <c r="I62" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D63" s="13"/>
+      <c r="E63" s="13"/>
+      <c r="F63" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G63" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" s="14"/>
+      <c r="I63" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C64" s="12"/>
+      <c r="D64" s="13"/>
+      <c r="E64" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F64" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G64" s="12"/>
+      <c r="H64" s="14"/>
+      <c r="I64" s="11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C65" s="8"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F65" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G65" s="8"/>
+      <c r="H65" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="I65" s="11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="14"/>
+      <c r="B66" s="14"/>
+      <c r="C66" s="12"/>
+      <c r="D66" s="13"/>
+      <c r="E66" s="13"/>
+      <c r="F66" s="13"/>
+      <c r="G66" s="12"/>
+      <c r="H66" s="14"/>
+      <c r="I66" s="15"/>
+    </row>
+    <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C67" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D67" s="13"/>
+      <c r="E67" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F67" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G67" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H67" s="14"/>
+      <c r="I67" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D68" s="13"/>
+      <c r="E68" s="13"/>
+      <c r="F68" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G68" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H68" s="14"/>
+      <c r="I68" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C69" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D69" s="13"/>
+      <c r="E69" s="13"/>
+      <c r="F69" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G69" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" s="14"/>
+      <c r="I69" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C70" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D70" s="13"/>
+      <c r="E70" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F70" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G70" s="12"/>
+      <c r="H70" s="14"/>
+      <c r="I70" s="11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D71" s="9"/>
+      <c r="E71" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F71" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G71" s="8"/>
+      <c r="H71" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="I71" s="11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="14"/>
+      <c r="B72" s="14"/>
+      <c r="C72" s="12"/>
+      <c r="D72" s="13"/>
+      <c r="E72" s="13"/>
+      <c r="F72" s="13"/>
+      <c r="G72" s="12"/>
+      <c r="H72" s="14"/>
+      <c r="I72" s="15"/>
+    </row>
+    <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="10"/>
+      <c r="B73" s="10"/>
+      <c r="C73" s="8"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="9"/>
+      <c r="F73" s="9"/>
+      <c r="G73" s="8"/>
+      <c r="H73" s="10"/>
+      <c r="I73" s="11"/>
+    </row>
+    <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="14"/>
+      <c r="B74" s="14"/>
+      <c r="C74" s="12"/>
+      <c r="D74" s="13"/>
+      <c r="E74" s="13"/>
+      <c r="F74" s="13"/>
+      <c r="G74" s="12"/>
+      <c r="H74" s="14"/>
+      <c r="I74" s="15"/>
+    </row>
+    <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="10"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="8"/>
+      <c r="D75" s="9"/>
+      <c r="E75" s="9"/>
+      <c r="F75" s="9"/>
+      <c r="G75" s="8"/>
+      <c r="H75" s="10"/>
+      <c r="I75" s="11"/>
+    </row>
+    <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="14"/>
+      <c r="B76" s="14"/>
+      <c r="C76" s="12"/>
+      <c r="D76" s="13"/>
+      <c r="E76" s="13"/>
+      <c r="F76" s="13"/>
+      <c r="G76" s="12"/>
+      <c r="H76" s="14"/>
+      <c r="I76" s="15"/>
+    </row>
+    <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="10"/>
+      <c r="B77" s="10"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="9"/>
+      <c r="E77" s="9"/>
+      <c r="F77" s="9"/>
+      <c r="G77" s="8"/>
+      <c r="H77" s="10"/>
+      <c r="I77" s="11"/>
+    </row>
+    <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="14"/>
+      <c r="B78" s="14"/>
+      <c r="C78" s="12"/>
+      <c r="D78" s="13"/>
+      <c r="E78" s="13"/>
+      <c r="F78" s="13"/>
+      <c r="G78" s="12"/>
+      <c r="H78" s="14"/>
+      <c r="I78" s="15"/>
+    </row>
+    <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="10"/>
+      <c r="B79" s="10"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="9"/>
+      <c r="E79" s="9"/>
+      <c r="F79" s="9"/>
+      <c r="G79" s="8"/>
+      <c r="H79" s="10"/>
+      <c r="I79" s="11"/>
+    </row>
+    <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="14"/>
+      <c r="B80" s="14"/>
+      <c r="C80" s="12"/>
+      <c r="D80" s="13"/>
+      <c r="E80" s="13"/>
+      <c r="F80" s="13"/>
+      <c r="G80" s="12"/>
+      <c r="H80" s="14"/>
+      <c r="I80" s="15"/>
+    </row>
+    <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="10"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="8"/>
+      <c r="D81" s="9"/>
+      <c r="E81" s="9"/>
+      <c r="F81" s="9"/>
+      <c r="G81" s="8"/>
+      <c r="H81" s="10"/>
+      <c r="I81" s="11"/>
+    </row>
+    <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="14"/>
+      <c r="B82" s="14"/>
+      <c r="C82" s="12"/>
+      <c r="D82" s="13"/>
+      <c r="E82" s="13"/>
+      <c r="F82" s="13"/>
+      <c r="G82" s="12"/>
+      <c r="H82" s="14"/>
+      <c r="I82" s="15"/>
+    </row>
+    <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="10"/>
+      <c r="B83" s="10"/>
+      <c r="C83" s="8"/>
+      <c r="D83" s="9"/>
+      <c r="E83" s="9"/>
+      <c r="F83" s="9"/>
+      <c r="G83" s="8"/>
+      <c r="H83" s="10"/>
+      <c r="I83" s="11"/>
+    </row>
+    <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="14"/>
+      <c r="B84" s="14"/>
+      <c r="C84" s="12"/>
+      <c r="D84" s="13"/>
+      <c r="E84" s="13"/>
+      <c r="F84" s="13"/>
+      <c r="G84" s="12"/>
+      <c r="H84" s="14"/>
+      <c r="I84" s="15"/>
+    </row>
+    <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="10"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="8"/>
+      <c r="D85" s="9"/>
+      <c r="E85" s="9"/>
+      <c r="F85" s="9"/>
+      <c r="G85" s="8"/>
+      <c r="H85" s="10"/>
+      <c r="I85" s="11"/>
+    </row>
+    <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="14"/>
+      <c r="B86" s="14"/>
+      <c r="C86" s="12"/>
+      <c r="D86" s="13"/>
+      <c r="E86" s="13"/>
+      <c r="F86" s="13"/>
+      <c r="G86" s="12"/>
+      <c r="H86" s="14"/>
+      <c r="I86" s="15"/>
+    </row>
+    <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="10"/>
+      <c r="B87" s="10"/>
+      <c r="C87" s="8"/>
+      <c r="D87" s="9"/>
+      <c r="E87" s="9"/>
+      <c r="F87" s="9"/>
+      <c r="G87" s="8"/>
+      <c r="H87" s="10"/>
+      <c r="I87" s="11"/>
+    </row>
+    <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="14"/>
+      <c r="B88" s="14"/>
+      <c r="C88" s="12"/>
+      <c r="D88" s="13"/>
+      <c r="E88" s="13"/>
+      <c r="F88" s="13"/>
+      <c r="G88" s="12"/>
+      <c r="H88" s="14"/>
+      <c r="I88" s="15"/>
+    </row>
+    <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="10"/>
+      <c r="B89" s="10"/>
+      <c r="C89" s="8"/>
+      <c r="D89" s="9"/>
+      <c r="E89" s="9"/>
+      <c r="F89" s="9"/>
+      <c r="G89" s="8"/>
+      <c r="H89" s="10"/>
+      <c r="I89" s="11"/>
+    </row>
+    <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="14"/>
+      <c r="B90" s="14"/>
+      <c r="C90" s="12"/>
+      <c r="D90" s="13"/>
+      <c r="E90" s="13"/>
+      <c r="F90" s="13"/>
+      <c r="G90" s="12"/>
+      <c r="H90" s="14"/>
+      <c r="I90" s="15"/>
+    </row>
+    <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="10"/>
+      <c r="B91" s="10"/>
+      <c r="C91" s="8"/>
+      <c r="D91" s="9"/>
+      <c r="E91" s="9"/>
+      <c r="F91" s="9"/>
+      <c r="G91" s="8"/>
+      <c r="H91" s="10"/>
+      <c r="I91" s="11"/>
+    </row>
+    <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="14"/>
+      <c r="B92" s="14"/>
+      <c r="C92" s="12"/>
+      <c r="D92" s="13"/>
+      <c r="E92" s="13"/>
+      <c r="F92" s="13"/>
+      <c r="G92" s="12"/>
+      <c r="H92" s="14"/>
+      <c r="I92" s="15"/>
+    </row>
+    <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="10"/>
+      <c r="B93" s="10"/>
+      <c r="C93" s="8"/>
+      <c r="D93" s="9"/>
+      <c r="E93" s="9"/>
+      <c r="F93" s="9"/>
+      <c r="G93" s="8"/>
+      <c r="H93" s="10"/>
+      <c r="I93" s="11"/>
+    </row>
+    <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="14"/>
+      <c r="B94" s="14"/>
+      <c r="C94" s="12"/>
+      <c r="D94" s="13"/>
+      <c r="E94" s="13"/>
+      <c r="F94" s="13"/>
+      <c r="G94" s="12"/>
+      <c r="H94" s="14"/>
+      <c r="I94" s="15"/>
+    </row>
+    <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="10"/>
+      <c r="B95" s="10"/>
+      <c r="C95" s="8"/>
+      <c r="D95" s="9"/>
+      <c r="E95" s="9"/>
+      <c r="F95" s="9"/>
+      <c r="G95" s="8"/>
+      <c r="H95" s="10"/>
+      <c r="I95" s="11"/>
+    </row>
+    <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A96" s="14"/>
+      <c r="B96" s="14"/>
+      <c r="C96" s="12"/>
+      <c r="D96" s="13"/>
+      <c r="E96" s="13"/>
+      <c r="F96" s="13"/>
+      <c r="G96" s="12"/>
+      <c r="H96" s="14"/>
+      <c r="I96" s="15"/>
+    </row>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C96" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E96" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F96" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1661,89 +2653,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>43</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>44</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>46</v>
+      <c r="A4" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>48</v>
+      <c r="A5" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>50</v>
+      <c r="A6" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>52</v>
+      <c r="A7" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>54</v>
+      <c r="A8" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>56</v>
+      <c r="A9" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>58</v>
+      <c r="A10" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>60</v>
+      <c r="A11" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>62</v>
+      <c r="A12" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
-        <v>63</v>
+      <c r="A14" s="18" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1751,7 +2743,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>64</v>
+        <v>116</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>10</v>
@@ -1766,27 +2758,27 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>65</v>
+        <v>117</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>66</v>
+        <v>118</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>68</v>
+      <c r="A17" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>120</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>20</v>
@@ -1795,160 +2787,160 @@
         <v>21</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>72</v>
+        <v>122</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>73</v>
+      <c r="A18" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>125</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>75</v>
+        <v>127</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>76</v>
+        <v>128</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>77</v>
+        <v>123</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>78</v>
+      <c r="A19" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>76</v>
+        <v>128</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>79</v>
+        <v>123</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>80</v>
+      <c r="A20" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>131</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>71</v>
+        <v>123</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>76</v>
+        <v>128</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>82</v>
+        <v>123</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>83</v>
+      <c r="A21" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>133</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>75</v>
+        <v>127</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>76</v>
+        <v>128</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="H21" s="11" t="s">
-        <v>86</v>
+        <v>134</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>87</v>
+      <c r="A22" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>136</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>90</v>
+        <v>123</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>87</v>
+      <c r="A23" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>136</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>20</v>
@@ -1957,65 +2949,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="H23" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="I23" s="14" t="s">
-        <v>92</v>
+        <v>122</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>93</v>
+      <c r="A24" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>141</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>76</v>
+        <v>128</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>95</v>
+        <v>123</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>96</v>
+      <c r="A25" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>144</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>76</v>
+        <v>128</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>99</v>
+        <v>146</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2045,15 +3037,15 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>100</v>
+        <v>148</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>21</v>
@@ -2061,23 +3053,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>101</v>
+        <v>149</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>102</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>103</v>
+        <v>151</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>76</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>104</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2087,27 +3079,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>105</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>81</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>106</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>107</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>108</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
criar modelo lógico e tabelas no DDL
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="157">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -126,298 +126,298 @@
     <t xml:space="preserve">data_admissao</t>
   </si>
   <si>
+    <t xml:space="preserve">Campo da data de admissão do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">função</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da Função do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matrícula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da Matrícula do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e-mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de E-mail do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do CPF do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">telefone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de telefone do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">senha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de senha do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação da função</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do nome da função</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do Nome do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de telefone do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECK(1,3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação da situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de E-mail do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">endereco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de endereço do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do Nome do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARCA / ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação da marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MODELO / ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação do modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIPO / ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Estrangeira de identificação do tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_emissão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_situação </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação da situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do Nome da situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_funcionario_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como preencher o Dicionário de Dados e Exemplo Demonstrativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Nome da Tabela:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identificador da tabela em minúsculas/snake_case (ex: alunos, cursos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Nome do Campo:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome exato da coluna no banco de dados (ex: id_aluno, cpf, data_nascimento).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Tipo de Dado:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo do atributo no SGBD (ex: INT, VARCHAR, DECIMAL, DATE). Use a lista suspensa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Tamanho / Precisão:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho do campo, se aplicável (ex: 100 para VARCHAR, 10,2 para DECIMAL).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Chave (PK/FK):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informe se o campo é Chave Primária (PK), Chave Estrangeira (FK), ou Ambos (PFK).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Permite Nulo?:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selecione SIM se aceitar valores nulos (NULL) ou NÃO se for NOT NULL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Valor Padrão:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor atribuído automaticamente caso nenhum seja informado (ex: CURRENT_TIMESTAMP, 0, 'ATIVO').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Tabela Referenciada:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso seja FK, informe a tabela e campo de origem (ex: cursos(id_curso)).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Descrição / Regra:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explicação clara do significado do dado e eventuais restrições ou regras de negócio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exemplo Preenchido:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome do Campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor Padrão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabela / Campo Referenciado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tb_alunos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_aluno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTO_INCREMENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identificador único do aluno.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_completo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VARCHAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nenhum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome civil completo do aluno.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apenas números. Deve ser único (UNIQUE).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_nascimento</t>
+  </si>
+  <si>
     <t xml:space="preserve">DATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo da data de admissão do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">função</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo da Função do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matrícula</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo da Matrícula do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">e-mail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo de E-mail do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cpf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do CPF do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">telefone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo de telefone do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">senha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo de senha do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Primária de identificação da função</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_funcao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do nome da função</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Primária de identificação do cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do Nome do cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo de telefone do cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_cadastro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Estrangeira de identificação do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_funcionario_funcao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHECK(1,3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Estrangeira de identificação da situação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo de E-mail do cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">endereco</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo de endereço do cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Primária de identificação do equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do Nome do equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_marca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARCA / ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Estrangeira de identificação da marca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_modelo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MODELO / ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Estrangeira de identificação do modelo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_tipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO / ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Estrangeira de identificação do tipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_emissão</t>
-  </si>
-  <si>
-    <t xml:space="preserve">situação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_situação </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Primária de identificação da situação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_situação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do Nome da situação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_marca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do id_funcionario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do id_funcionario_funcao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modelo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_modelo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_tipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como preencher o Dicionário de Dados e Exemplo Demonstrativo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Nome da Tabela:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identificador da tabela em minúsculas/snake_case (ex: alunos, cursos).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Nome do Campo:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome exato da coluna no banco de dados (ex: id_aluno, cpf, data_nascimento).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Tipo de Dado:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo do atributo no SGBD (ex: INT, VARCHAR, DECIMAL, DATE). Use a lista suspensa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Tamanho / Precisão:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tamanho do campo, se aplicável (ex: 100 para VARCHAR, 10,2 para DECIMAL).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Chave (PK/FK):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Informe se o campo é Chave Primária (PK), Chave Estrangeira (FK), ou Ambos (PFK).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Permite Nulo?:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Selecione SIM se aceitar valores nulos (NULL) ou NÃO se for NOT NULL.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Valor Padrão:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor atribuído automaticamente caso nenhum seja informado (ex: CURRENT_TIMESTAMP, 0, 'ATIVO').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8. Tabela Referenciada:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caso seja FK, informe a tabela e campo de origem (ex: cursos(id_curso)).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9. Descrição / Regra:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explicação clara do significado do dado e eventuais restrições ou regras de negócio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exemplo Preenchido:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome do Campo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor Padrão</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tabela / Campo Referenciado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tb_alunos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_aluno</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTO_INCREMENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identificador único do aluno.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_completo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VARCHAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nenhum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome civil completo do aluno.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apenas números. Deve ser único (UNIQUE).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_nascimento</t>
   </si>
   <si>
     <t xml:space="preserve">Data de nascimento para cálculo de idade.</t>
@@ -1165,7 +1165,7 @@
         <v>33</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
@@ -1175,7 +1175,7 @@
       <c r="G14" s="12"/>
       <c r="H14" s="14"/>
       <c r="I14" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1183,7 +1183,7 @@
         <v>17</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>25</v>
@@ -1196,7 +1196,7 @@
       <c r="G15" s="12"/>
       <c r="H15" s="14"/>
       <c r="I15" s="15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1204,7 +1204,7 @@
         <v>17</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>25</v>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="H16" s="14"/>
       <c r="I16" s="15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1227,7 +1227,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>25</v>
@@ -1235,12 +1235,12 @@
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
       <c r="F17" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G17" s="12"/>
       <c r="H17" s="14"/>
       <c r="I17" s="15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1248,7 +1248,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>25</v>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="H18" s="14"/>
       <c r="I18" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1271,7 +1271,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C19" s="12" t="s">
         <v>25</v>
@@ -1279,12 +1279,12 @@
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
       <c r="F19" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G19" s="12"/>
       <c r="H19" s="14"/>
       <c r="I19" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1292,7 +1292,7 @@
         <v>17</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>25</v>
@@ -1305,7 +1305,7 @@
       <c r="G20" s="12"/>
       <c r="H20" s="14"/>
       <c r="I20" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1321,7 +1321,7 @@
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>27</v>
@@ -1341,15 +1341,15 @@
       </c>
       <c r="H22" s="14"/>
       <c r="I22" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>25</v>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="H23" s="14"/>
       <c r="I23" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>31</v>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="H24" s="14"/>
       <c r="I24" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1414,10 +1414,10 @@
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>54</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>19</v>
@@ -1434,15 +1434,15 @@
       </c>
       <c r="H27" s="10"/>
       <c r="I27" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C28" s="12" t="s">
         <v>25</v>
@@ -1455,15 +1455,15 @@
       <c r="G28" s="12"/>
       <c r="H28" s="14"/>
       <c r="I28" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>25</v>
@@ -1474,17 +1474,19 @@
         <v>21</v>
       </c>
       <c r="G29" s="12"/>
-      <c r="H29" s="14"/>
+      <c r="H29" s="14" t="s">
+        <v>29</v>
+      </c>
       <c r="I29" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="13"/>
@@ -1496,7 +1498,7 @@
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>18</v>
@@ -1514,15 +1516,15 @@
       <c r="G31" s="12"/>
       <c r="H31" s="14"/>
       <c r="I31" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>19</v>
@@ -1536,15 +1538,15 @@
       </c>
       <c r="G32" s="12"/>
       <c r="H32" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>31</v>
@@ -1562,15 +1564,15 @@
       <c r="G33" s="12"/>
       <c r="H33" s="14"/>
       <c r="I33" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>25</v>
@@ -1585,15 +1587,15 @@
       </c>
       <c r="H34" s="14"/>
       <c r="I34" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" s="12" t="s">
         <v>25</v>
@@ -1601,20 +1603,20 @@
       <c r="D35" s="13"/>
       <c r="E35" s="13"/>
       <c r="F35" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G35" s="12"/>
       <c r="H35" s="14"/>
       <c r="I35" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C36" s="12" t="s">
         <v>25</v>
@@ -1622,12 +1624,12 @@
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
       <c r="F36" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G36" s="12"/>
       <c r="H36" s="14"/>
       <c r="I36" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1665,10 +1667,10 @@
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>19</v>
@@ -1685,15 +1687,15 @@
       </c>
       <c r="H40" s="10"/>
       <c r="I40" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C41" s="12" t="s">
         <v>25</v>
@@ -1706,15 +1708,15 @@
       <c r="G41" s="12"/>
       <c r="H41" s="14"/>
       <c r="I41" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C42" s="12" t="s">
         <v>19</v>
@@ -1726,18 +1728,18 @@
       <c r="F42" s="13"/>
       <c r="G42" s="12"/>
       <c r="H42" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="I42" s="11" t="s">
         <v>72</v>
-      </c>
-      <c r="I42" s="11" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>19</v>
@@ -1749,18 +1751,18 @@
       <c r="F43" s="13"/>
       <c r="G43" s="12"/>
       <c r="H43" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="I43" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="I43" s="11" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C44" s="12" t="s">
         <v>19</v>
@@ -1772,18 +1774,18 @@
       <c r="F44" s="13"/>
       <c r="G44" s="12"/>
       <c r="H44" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="I44" s="11" t="s">
         <v>78</v>
-      </c>
-      <c r="I44" s="11" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C45" s="12" t="s">
         <v>19</v>
@@ -1801,7 +1803,7 @@
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B46" s="7" t="s">
         <v>31</v>
@@ -1822,10 +1824,10 @@
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C47" s="12" t="s">
         <v>25</v>
@@ -1863,10 +1865,10 @@
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B50" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="B50" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>19</v>
@@ -1883,15 +1885,15 @@
       </c>
       <c r="H50" s="10"/>
       <c r="I50" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C51" s="12" t="s">
         <v>25</v>
@@ -1904,15 +1906,15 @@
       <c r="G51" s="12"/>
       <c r="H51" s="14"/>
       <c r="I51" s="15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>25</v>
@@ -1928,7 +1930,7 @@
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B53" s="7" t="s">
         <v>31</v>
@@ -1958,10 +1960,10 @@
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C55" s="12" t="s">
         <v>19</v>
@@ -1978,15 +1980,15 @@
       </c>
       <c r="H55" s="14"/>
       <c r="I55" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B56" s="7" t="s">
         <v>87</v>
-      </c>
-      <c r="B56" s="7" t="s">
-        <v>88</v>
       </c>
       <c r="C56" s="12" t="s">
         <v>25</v>
@@ -2001,12 +2003,12 @@
       </c>
       <c r="H56" s="14"/>
       <c r="I56" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>31</v>
@@ -2024,12 +2026,12 @@
       </c>
       <c r="H57" s="14"/>
       <c r="I57" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B58" s="7" t="s">
         <v>18</v>
@@ -2045,15 +2047,15 @@
       <c r="G58" s="12"/>
       <c r="H58" s="14"/>
       <c r="I58" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
@@ -2065,10 +2067,10 @@
       </c>
       <c r="G59" s="8"/>
       <c r="H59" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2084,10 +2086,10 @@
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C61" s="12" t="s">
         <v>19</v>
@@ -2104,15 +2106,15 @@
       </c>
       <c r="H61" s="14"/>
       <c r="I61" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62" s="7" t="s">
         <v>91</v>
-      </c>
-      <c r="B62" s="7" t="s">
-        <v>92</v>
       </c>
       <c r="C62" s="12" t="s">
         <v>25</v>
@@ -2127,12 +2129,12 @@
       </c>
       <c r="H62" s="14"/>
       <c r="I62" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B63" s="7" t="s">
         <v>31</v>
@@ -2150,12 +2152,12 @@
       </c>
       <c r="H63" s="14"/>
       <c r="I63" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B64" s="7" t="s">
         <v>18</v>
@@ -2171,15 +2173,15 @@
       <c r="G64" s="12"/>
       <c r="H64" s="14"/>
       <c r="I64" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
@@ -2191,10 +2193,10 @@
       </c>
       <c r="G65" s="8"/>
       <c r="H65" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2210,10 +2212,10 @@
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C67" s="12" t="s">
         <v>19</v>
@@ -2230,15 +2232,15 @@
       </c>
       <c r="H67" s="14"/>
       <c r="I67" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B68" s="7" t="s">
         <v>93</v>
-      </c>
-      <c r="B68" s="7" t="s">
-        <v>94</v>
       </c>
       <c r="C68" s="12" t="s">
         <v>25</v>
@@ -2253,12 +2255,12 @@
       </c>
       <c r="H68" s="14"/>
       <c r="I68" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B69" s="7" t="s">
         <v>31</v>
@@ -2276,12 +2278,12 @@
       </c>
       <c r="H69" s="14"/>
       <c r="I69" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B70" s="7" t="s">
         <v>18</v>
@@ -2299,15 +2301,15 @@
       <c r="G70" s="12"/>
       <c r="H70" s="14"/>
       <c r="I70" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C71" s="12" t="s">
         <v>19</v>
@@ -2321,10 +2323,10 @@
       </c>
       <c r="G71" s="8"/>
       <c r="H71" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2653,89 +2655,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="17" t="s">
         <v>97</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>99</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B6" s="17" t="s">
         <v>101</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>103</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="17" t="s">
         <v>105</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>107</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>109</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>111</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" s="17" t="s">
         <v>113</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2743,7 +2745,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>10</v>
@@ -2758,10 +2760,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>118</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>16</v>
@@ -2769,16 +2771,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>119</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>120</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>20</v>
@@ -2787,88 +2789,88 @@
         <v>21</v>
       </c>
       <c r="G17" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="H17" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="H17" s="14" t="s">
+      <c r="I17" s="15" t="s">
         <v>123</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B18" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="D18" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="E18" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="F18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="H18" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B20" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>34</v>
-      </c>
       <c r="D20" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>132</v>
@@ -2876,22 +2878,22 @@
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>133</v>
       </c>
       <c r="C21" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="E21" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="E21" s="13" t="s">
-        <v>128</v>
-      </c>
       <c r="F21" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G21" s="12" t="s">
         <v>134</v>
@@ -2902,7 +2904,7 @@
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>136</v>
@@ -2911,7 +2913,7 @@
         <v>19</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>28</v>
@@ -2920,7 +2922,7 @@
         <v>21</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>137</v>
@@ -2940,7 +2942,7 @@
         <v>19</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>20</v>
@@ -2949,10 +2951,10 @@
         <v>21</v>
       </c>
       <c r="G23" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="H23" s="14" t="s">
         <v>122</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>123</v>
       </c>
       <c r="I23" s="15" t="s">
         <v>140</v>
@@ -2966,19 +2968,19 @@
         <v>141</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>142</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>143</v>
@@ -2998,7 +3000,7 @@
         <v>145</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>21</v>
@@ -3037,7 +3039,7 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3064,7 +3066,7 @@
         <v>151</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3084,7 +3086,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>34</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
iniciar tabela ordem de servicos dbeaver e draw.io
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="158">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t xml:space="preserve">nome_tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem serviço</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -2341,7 +2344,9 @@
       <c r="I72" s="15"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="10"/>
+      <c r="A73" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B73" s="10"/>
       <c r="C73" s="8"/>
       <c r="D73" s="9"/>
@@ -2352,7 +2357,9 @@
       <c r="I73" s="11"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="14"/>
+      <c r="A74" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B74" s="14"/>
       <c r="C74" s="12"/>
       <c r="D74" s="13"/>
@@ -2363,7 +2370,9 @@
       <c r="I74" s="15"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="10"/>
+      <c r="A75" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B75" s="10"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
@@ -2374,7 +2383,9 @@
       <c r="I75" s="11"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="14"/>
+      <c r="A76" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B76" s="14"/>
       <c r="C76" s="12"/>
       <c r="D76" s="13"/>
@@ -2385,7 +2396,9 @@
       <c r="I76" s="15"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="10"/>
+      <c r="A77" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B77" s="10"/>
       <c r="C77" s="8"/>
       <c r="D77" s="9"/>
@@ -2396,7 +2409,9 @@
       <c r="I77" s="11"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="14"/>
+      <c r="A78" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B78" s="14"/>
       <c r="C78" s="12"/>
       <c r="D78" s="13"/>
@@ -2407,7 +2422,9 @@
       <c r="I78" s="15"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="10"/>
+      <c r="A79" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B79" s="10"/>
       <c r="C79" s="8"/>
       <c r="D79" s="9"/>
@@ -2418,7 +2435,9 @@
       <c r="I79" s="11"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="14"/>
+      <c r="A80" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B80" s="14"/>
       <c r="C80" s="12"/>
       <c r="D80" s="13"/>
@@ -2429,7 +2448,9 @@
       <c r="I80" s="15"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="10"/>
+      <c r="A81" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B81" s="10"/>
       <c r="C81" s="8"/>
       <c r="D81" s="9"/>
@@ -2440,7 +2461,9 @@
       <c r="I81" s="11"/>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="14"/>
+      <c r="A82" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B82" s="14"/>
       <c r="C82" s="12"/>
       <c r="D82" s="13"/>
@@ -2451,7 +2474,9 @@
       <c r="I82" s="15"/>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="10"/>
+      <c r="A83" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B83" s="10"/>
       <c r="C83" s="8"/>
       <c r="D83" s="9"/>
@@ -2462,7 +2487,9 @@
       <c r="I83" s="11"/>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="14"/>
+      <c r="A84" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B84" s="14"/>
       <c r="C84" s="12"/>
       <c r="D84" s="13"/>
@@ -2473,7 +2500,9 @@
       <c r="I84" s="15"/>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="10"/>
+      <c r="A85" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B85" s="10"/>
       <c r="C85" s="8"/>
       <c r="D85" s="9"/>
@@ -2484,7 +2513,9 @@
       <c r="I85" s="11"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="14"/>
+      <c r="A86" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B86" s="14"/>
       <c r="C86" s="12"/>
       <c r="D86" s="13"/>
@@ -2655,89 +2686,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2745,7 +2776,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>10</v>
@@ -2760,10 +2791,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>16</v>
@@ -2771,16 +2802,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>20</v>
@@ -2789,131 +2820,131 @@
         <v>21</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H17" s="14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>40</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>28</v>
@@ -2922,27 +2953,27 @@
         <v>21</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>20</v>
@@ -2951,65 +2982,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -3044,7 +3075,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>28</v>
@@ -3055,23 +3086,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3081,27 +3112,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
criar tabelas pecas - servicos - categoria
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -10,7 +10,7 @@
   <sheets>
     <sheet name="Dicionário de Dados" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Instruções e Exemplo" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Validações" sheetId="3" state="hidden" r:id="rId5"/>
+    <sheet name="Validações" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="214">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -183,7 +183,7 @@
     <t xml:space="preserve">cliente</t>
   </si>
   <si>
-    <t xml:space="preserve">id </t>
+    <t xml:space="preserve">id_cliente </t>
   </si>
   <si>
     <t xml:space="preserve">Chave Primária de identificação do cliente</t>
@@ -225,6 +225,9 @@
     <t xml:space="preserve">equipamento</t>
   </si>
   <si>
+    <t xml:space="preserve">id_equipamento</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chave Primária de identificação do equipamento</t>
   </si>
   <si>
@@ -282,12 +285,21 @@
     <t xml:space="preserve">Campo do Nome da situação</t>
   </si>
   <si>
+    <t xml:space="preserve">Campo do Nome da data de emissão</t>
+  </si>
+  <si>
     <t xml:space="preserve">marca</t>
   </si>
   <si>
+    <t xml:space="preserve">Chave Primária de identificação da marca</t>
+  </si>
+  <si>
     <t xml:space="preserve">nome_marca</t>
   </si>
   <si>
+    <t xml:space="preserve">Campo do nome da marca</t>
+  </si>
+  <si>
     <t xml:space="preserve">Campo do id_funcionario</t>
   </si>
   <si>
@@ -297,16 +309,172 @@
     <t xml:space="preserve">modelo</t>
   </si>
   <si>
+    <t xml:space="preserve">Chave Primária de identificação do modelo</t>
+  </si>
+  <si>
     <t xml:space="preserve">nome_modelo</t>
   </si>
   <si>
+    <t xml:space="preserve">Campo do nome do modelo</t>
+  </si>
+  <si>
     <t xml:space="preserve">tipo</t>
   </si>
   <si>
+    <t xml:space="preserve">Chave Primária de identificação do tipo</t>
+  </si>
+  <si>
     <t xml:space="preserve">nome_tipo</t>
   </si>
   <si>
+    <t xml:space="preserve">Campo do nome do tipo</t>
+  </si>
+  <si>
     <t xml:space="preserve">ordem serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_ordem_serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação da ordem de serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_funcionario_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_funcao_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_funcionario_funcao_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da data_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_fechamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da data_fechamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_status_atual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do status atual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">descricacao_defeito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da descrição_defeito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">defeito_constatado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do defeito_constatado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do valor total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tecnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_tecnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tecnico_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id_tecnico_funcao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peças</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_pecas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_peças</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do nome das peças</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco_base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do preço base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horas_trabalho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo horas de trabalho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">serviços</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_serviços</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_serviços</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do nome de serviços</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do id da categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do preço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo das horas de trabalho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da data de emissão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo nome da categoria</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -655,13 +823,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -696,10 +868,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -712,12 +880,28 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -988,112 +1172,112 @@
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="33.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5"/>
+      <c r="B4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5"/>
+      <c r="B5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9" t="s">
+      <c r="C10" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="8" t="s">
+      <c r="F10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="10"/>
+      <c r="H10" s="9"/>
       <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="12" t="s">
@@ -1105,16 +1289,16 @@
         <v>21</v>
       </c>
       <c r="G11" s="12"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="s">
+      <c r="H11" s="12"/>
+      <c r="I11" s="14" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="12" t="s">
@@ -1138,10 +1322,10 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C13" s="12" t="s">
@@ -1155,16 +1339,16 @@
       <c r="G13" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="14"/>
+      <c r="H13" s="12"/>
       <c r="I13" s="11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>33</v>
       </c>
       <c r="C14" s="12" t="s">
@@ -1176,16 +1360,16 @@
         <v>21</v>
       </c>
       <c r="G14" s="12"/>
-      <c r="H14" s="14"/>
+      <c r="H14" s="12"/>
       <c r="I14" s="11" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="16" t="s">
         <v>35</v>
       </c>
       <c r="C15" s="12" t="s">
@@ -1197,16 +1381,16 @@
         <v>21</v>
       </c>
       <c r="G15" s="12"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="s">
+      <c r="H15" s="12"/>
+      <c r="I15" s="14" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="16" t="s">
         <v>37</v>
       </c>
       <c r="C16" s="12" t="s">
@@ -1220,16 +1404,16 @@
       <c r="G16" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="s">
+      <c r="H16" s="12"/>
+      <c r="I16" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="16" t="s">
         <v>39</v>
       </c>
       <c r="C17" s="12" t="s">
@@ -1241,16 +1425,16 @@
         <v>40</v>
       </c>
       <c r="G17" s="12"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="s">
+      <c r="H17" s="12"/>
+      <c r="I17" s="14" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C18" s="12" t="s">
@@ -1264,16 +1448,16 @@
       <c r="G18" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="s">
+      <c r="H18" s="12"/>
+      <c r="I18" s="14" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="16" t="s">
         <v>44</v>
       </c>
       <c r="C19" s="12" t="s">
@@ -1285,16 +1469,16 @@
         <v>40</v>
       </c>
       <c r="G19" s="12"/>
-      <c r="H19" s="14"/>
+      <c r="H19" s="12"/>
       <c r="I19" s="11" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="16" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="12" t="s">
@@ -1306,27 +1490,27 @@
         <v>21</v>
       </c>
       <c r="G20" s="12"/>
-      <c r="H20" s="14"/>
+      <c r="H20" s="12"/>
       <c r="I20" s="11" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10"/>
-      <c r="B21" s="14"/>
+      <c r="A21" s="15"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="12"/>
       <c r="D21" s="13"/>
       <c r="E21" s="13"/>
       <c r="F21" s="13"/>
       <c r="G21" s="12"/>
-      <c r="H21" s="14"/>
+      <c r="H21" s="12"/>
       <c r="I21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C22" s="12" t="s">
@@ -1342,16 +1526,16 @@
       <c r="G22" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H22" s="14"/>
+      <c r="H22" s="12"/>
       <c r="I22" s="11" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="8" t="s">
         <v>49</v>
       </c>
       <c r="C23" s="12" t="s">
@@ -1365,16 +1549,16 @@
       <c r="G23" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H23" s="14"/>
+      <c r="H23" s="12"/>
       <c r="I23" s="11" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C24" s="12" t="s">
@@ -1388,63 +1572,63 @@
       <c r="G24" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="14"/>
+      <c r="H24" s="12"/>
       <c r="I24" s="11" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10"/>
-      <c r="B25" s="14"/>
+      <c r="A25" s="15"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="12"/>
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
       <c r="F25" s="13"/>
       <c r="G25" s="12"/>
-      <c r="H25" s="14"/>
+      <c r="H25" s="12"/>
       <c r="I25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10"/>
-      <c r="B26" s="14"/>
+      <c r="A26" s="15"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="12"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
       <c r="G26" s="12"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C27" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9" t="s">
+      <c r="C27" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G27" s="8" t="s">
+      <c r="F27" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H27" s="10"/>
+      <c r="H27" s="9"/>
       <c r="I27" s="11" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>55</v>
       </c>
       <c r="C28" s="12" t="s">
@@ -1456,16 +1640,16 @@
         <v>21</v>
       </c>
       <c r="G28" s="12"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="s">
+      <c r="H28" s="12"/>
+      <c r="I28" s="14" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
         <v>39</v>
       </c>
       <c r="C29" s="12" t="s">
@@ -1477,7 +1661,7 @@
         <v>21</v>
       </c>
       <c r="G29" s="12"/>
-      <c r="H29" s="14" t="s">
+      <c r="H29" s="12" t="s">
         <v>29</v>
       </c>
       <c r="I29" s="11" t="s">
@@ -1485,10 +1669,10 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="8" t="s">
         <v>58</v>
       </c>
       <c r="C30" s="12"/>
@@ -1496,14 +1680,14 @@
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
       <c r="G30" s="12"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="14"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C31" s="12" t="s">
@@ -1517,16 +1701,16 @@
         <v>21</v>
       </c>
       <c r="G31" s="12"/>
-      <c r="H31" s="14"/>
+      <c r="H31" s="12"/>
       <c r="I31" s="11" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="8" t="s">
         <v>60</v>
       </c>
       <c r="C32" s="12" t="s">
@@ -1540,7 +1724,7 @@
         <v>21</v>
       </c>
       <c r="G32" s="12"/>
-      <c r="H32" s="14" t="s">
+      <c r="H32" s="12" t="s">
         <v>61</v>
       </c>
       <c r="I32" s="11" t="s">
@@ -1548,10 +1732,10 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
@@ -1565,16 +1749,16 @@
         <v>21</v>
       </c>
       <c r="G33" s="12"/>
-      <c r="H33" s="14"/>
+      <c r="H33" s="12"/>
       <c r="I33" s="11" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="14" t="s">
+      <c r="A34" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C34" s="12" t="s">
@@ -1588,16 +1772,16 @@
       <c r="G34" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="s">
+      <c r="H34" s="12"/>
+      <c r="I34" s="14" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14" t="s">
+      <c r="A35" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="16" t="s">
         <v>39</v>
       </c>
       <c r="C35" s="12" t="s">
@@ -1609,16 +1793,16 @@
         <v>40</v>
       </c>
       <c r="G35" s="12"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="s">
+      <c r="H35" s="12"/>
+      <c r="I35" s="14" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="s">
+      <c r="A36" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="16" t="s">
         <v>64</v>
       </c>
       <c r="C36" s="12" t="s">
@@ -1630,75 +1814,75 @@
         <v>40</v>
       </c>
       <c r="G36" s="12"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="s">
+      <c r="H36" s="12"/>
+      <c r="I36" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
       <c r="C37" s="12"/>
       <c r="D37" s="13"/>
       <c r="E37" s="13"/>
       <c r="F37" s="13"/>
       <c r="G37" s="12"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="14"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14"/>
+      <c r="A38" s="16"/>
+      <c r="B38" s="16"/>
       <c r="C38" s="12"/>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
       <c r="F38" s="13"/>
       <c r="G38" s="12"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="14"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14"/>
-      <c r="B39" s="14"/>
+      <c r="A39" s="16"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="12"/>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
       <c r="G39" s="12"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="14"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B40" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9" t="s">
+      <c r="B40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F40" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G40" s="8" t="s">
+      <c r="F40" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H40" s="10"/>
+      <c r="H40" s="9"/>
       <c r="I40" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
+      <c r="A41" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B41" s="7" t="s">
-        <v>68</v>
+      <c r="B41" s="8" t="s">
+        <v>69</v>
       </c>
       <c r="C41" s="12" t="s">
         <v>25</v>
@@ -1709,17 +1893,17 @@
         <v>21</v>
       </c>
       <c r="G41" s="12"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="s">
-        <v>69</v>
+      <c r="H41" s="12"/>
+      <c r="I41" s="14" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
+      <c r="A42" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>70</v>
+      <c r="B42" s="8" t="s">
+        <v>71</v>
       </c>
       <c r="C42" s="12" t="s">
         <v>19</v>
@@ -1730,19 +1914,19 @@
       </c>
       <c r="F42" s="13"/>
       <c r="G42" s="12"/>
-      <c r="H42" s="14" t="s">
-        <v>71</v>
+      <c r="H42" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="s">
+      <c r="A43" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B43" s="7" t="s">
-        <v>73</v>
+      <c r="B43" s="8" t="s">
+        <v>74</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>19</v>
@@ -1753,19 +1937,19 @@
       </c>
       <c r="F43" s="13"/>
       <c r="G43" s="12"/>
-      <c r="H43" s="14" t="s">
-        <v>74</v>
+      <c r="H43" s="12" t="s">
+        <v>75</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="s">
+      <c r="A44" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B44" s="7" t="s">
-        <v>76</v>
+      <c r="B44" s="8" t="s">
+        <v>77</v>
       </c>
       <c r="C44" s="12" t="s">
         <v>19</v>
@@ -1776,19 +1960,19 @@
       </c>
       <c r="F44" s="13"/>
       <c r="G44" s="12"/>
-      <c r="H44" s="14" t="s">
-        <v>77</v>
+      <c r="H44" s="12" t="s">
+        <v>78</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="s">
+      <c r="A45" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B45" s="7" t="s">
-        <v>79</v>
+      <c r="B45" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="C45" s="12" t="s">
         <v>19</v>
@@ -1801,14 +1985,14 @@
         <v>21</v>
       </c>
       <c r="G45" s="12"/>
-      <c r="H45" s="14"/>
+      <c r="H45" s="12"/>
       <c r="I45" s="11"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="s">
+      <c r="A46" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="B46" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C46" s="12" t="s">
@@ -1822,15 +2006,15 @@
       <c r="G46" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H46" s="14"/>
+      <c r="H46" s="12"/>
       <c r="I46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
+      <c r="A47" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B47" s="7" t="s">
-        <v>80</v>
+      <c r="B47" s="8" t="s">
+        <v>81</v>
       </c>
       <c r="C47" s="12" t="s">
         <v>25</v>
@@ -1841,62 +2025,62 @@
         <v>21</v>
       </c>
       <c r="G47" s="12"/>
-      <c r="H47" s="14"/>
+      <c r="H47" s="12"/>
       <c r="I47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="14"/>
-      <c r="B48" s="14"/>
+      <c r="A48" s="16"/>
+      <c r="B48" s="16"/>
       <c r="C48" s="12"/>
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
       <c r="F48" s="13"/>
       <c r="G48" s="12"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15"/>
+      <c r="H48" s="12"/>
+      <c r="I48" s="14"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="14"/>
-      <c r="B49" s="14"/>
+      <c r="A49" s="16"/>
+      <c r="B49" s="16"/>
       <c r="C49" s="12"/>
       <c r="D49" s="13"/>
       <c r="E49" s="13"/>
       <c r="F49" s="13"/>
       <c r="G49" s="12"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15"/>
+      <c r="H49" s="12"/>
+      <c r="I49" s="14"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="B50" s="7" t="s">
+      <c r="A50" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="C50" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9" t="s">
+      <c r="B50" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F50" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G50" s="8" t="s">
+      <c r="F50" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G50" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H50" s="10"/>
+      <c r="H50" s="9"/>
       <c r="I50" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="B51" s="7" t="s">
-        <v>84</v>
+      <c r="A51" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>85</v>
       </c>
       <c r="C51" s="12" t="s">
         <v>25</v>
@@ -1907,35 +2091,37 @@
         <v>21</v>
       </c>
       <c r="G51" s="12"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="s">
-        <v>85</v>
+      <c r="H51" s="12"/>
+      <c r="I51" s="14" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="s">
+      <c r="A52" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B52" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B52" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C52" s="8" t="s">
+      <c r="C52" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G52" s="8"/>
-      <c r="H52" s="10"/>
-      <c r="I52" s="11"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
+      <c r="I52" s="14" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="B53" s="7" t="s">
+      <c r="A53" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B53" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C53" s="12" t="s">
@@ -1947,26 +2133,28 @@
         <v>21</v>
       </c>
       <c r="G53" s="12"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15"/>
+      <c r="H53" s="12"/>
+      <c r="I53" s="14" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="10"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="10"/>
+      <c r="A54" s="15"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="10"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="10"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="9"/>
       <c r="I54" s="11"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B55" s="7" t="s">
-        <v>70</v>
+      <c r="A55" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>71</v>
       </c>
       <c r="C55" s="12" t="s">
         <v>19</v>
@@ -1981,17 +2169,17 @@
       <c r="G55" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H55" s="14"/>
+      <c r="H55" s="12"/>
       <c r="I55" s="11" t="s">
-        <v>48</v>
+        <v>89</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B56" s="7" t="s">
-        <v>87</v>
+      <c r="A56" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>90</v>
       </c>
       <c r="C56" s="12" t="s">
         <v>25</v>
@@ -2004,16 +2192,16 @@
       <c r="G56" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H56" s="14"/>
+      <c r="H56" s="12"/>
       <c r="I56" s="11" t="s">
-        <v>50</v>
+        <v>91</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B57" s="7" t="s">
+      <c r="A57" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B57" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C57" s="12" t="s">
@@ -2027,16 +2215,16 @@
       <c r="G57" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H57" s="14"/>
+      <c r="H57" s="12"/>
       <c r="I57" s="11" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B58" s="7" t="s">
+      <c r="A58" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C58" s="12"/>
@@ -2048,51 +2236,51 @@
         <v>21</v>
       </c>
       <c r="G58" s="12"/>
-      <c r="H58" s="14"/>
+      <c r="H58" s="12"/>
       <c r="I58" s="11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="8" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B59" s="7" t="s">
+      <c r="B59" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C59" s="8"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9" t="s">
+      <c r="C59" s="9"/>
+      <c r="D59" s="10"/>
+      <c r="E59" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F59" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G59" s="8"/>
-      <c r="H59" s="10" t="s">
+      <c r="F59" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9" t="s">
         <v>61</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="14"/>
-      <c r="B60" s="14"/>
+      <c r="A60" s="16"/>
+      <c r="B60" s="16"/>
       <c r="C60" s="12"/>
       <c r="D60" s="13"/>
       <c r="E60" s="13"/>
       <c r="F60" s="13"/>
       <c r="G60" s="12"/>
-      <c r="H60" s="14"/>
-      <c r="I60" s="15"/>
+      <c r="H60" s="12"/>
+      <c r="I60" s="14"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B61" s="7" t="s">
-        <v>73</v>
+      <c r="A61" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>74</v>
       </c>
       <c r="C61" s="12" t="s">
         <v>19</v>
@@ -2107,17 +2295,17 @@
       <c r="G61" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H61" s="14"/>
+      <c r="H61" s="12"/>
       <c r="I61" s="11" t="s">
-        <v>48</v>
+        <v>95</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B62" s="7" t="s">
-        <v>91</v>
+      <c r="A62" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>96</v>
       </c>
       <c r="C62" s="12" t="s">
         <v>25</v>
@@ -2130,16 +2318,16 @@
       <c r="G62" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H62" s="14"/>
+      <c r="H62" s="12"/>
       <c r="I62" s="11" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B63" s="7" t="s">
+      <c r="A63" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B63" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C63" s="12" t="s">
@@ -2153,16 +2341,16 @@
       <c r="G63" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H63" s="14"/>
+      <c r="H63" s="12"/>
       <c r="I63" s="11" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B64" s="7" t="s">
+      <c r="A64" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B64" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C64" s="12"/>
@@ -2174,51 +2362,51 @@
         <v>21</v>
       </c>
       <c r="G64" s="12"/>
-      <c r="H64" s="14"/>
+      <c r="H64" s="12"/>
       <c r="I64" s="11" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B65" s="7" t="s">
+      <c r="A65" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B65" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C65" s="8"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9" t="s">
+      <c r="C65" s="9"/>
+      <c r="D65" s="10"/>
+      <c r="E65" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F65" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G65" s="8"/>
-      <c r="H65" s="10" t="s">
+      <c r="F65" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9" t="s">
         <v>61</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="14"/>
-      <c r="B66" s="14"/>
+      <c r="A66" s="16"/>
+      <c r="B66" s="16"/>
       <c r="C66" s="12"/>
       <c r="D66" s="13"/>
       <c r="E66" s="13"/>
       <c r="F66" s="13"/>
       <c r="G66" s="12"/>
-      <c r="H66" s="14"/>
-      <c r="I66" s="15"/>
+      <c r="H66" s="12"/>
+      <c r="I66" s="14"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B67" s="7" t="s">
-        <v>76</v>
+      <c r="A67" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>77</v>
       </c>
       <c r="C67" s="12" t="s">
         <v>19</v>
@@ -2233,17 +2421,17 @@
       <c r="G67" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H67" s="14"/>
+      <c r="H67" s="12"/>
       <c r="I67" s="11" t="s">
-        <v>48</v>
+        <v>99</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B68" s="7" t="s">
-        <v>93</v>
+      <c r="A68" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>100</v>
       </c>
       <c r="C68" s="12" t="s">
         <v>25</v>
@@ -2256,16 +2444,16 @@
       <c r="G68" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H68" s="14"/>
+      <c r="H68" s="12"/>
       <c r="I68" s="11" t="s">
-        <v>50</v>
+        <v>101</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B69" s="7" t="s">
+      <c r="A69" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B69" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C69" s="12" t="s">
@@ -2279,16 +2467,16 @@
       <c r="G69" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H69" s="14"/>
+      <c r="H69" s="12"/>
       <c r="I69" s="11" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B70" s="7" t="s">
+      <c r="A70" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C70" s="12" t="s">
@@ -2302,357 +2490,712 @@
         <v>21</v>
       </c>
       <c r="G70" s="12"/>
-      <c r="H70" s="14"/>
+      <c r="H70" s="12"/>
       <c r="I70" s="11" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B71" s="7" t="s">
+      <c r="A71" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71" s="8" t="s">
         <v>60</v>
       </c>
       <c r="C71" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D71" s="9"/>
-      <c r="E71" s="9" t="s">
+      <c r="D71" s="10"/>
+      <c r="E71" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F71" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G71" s="8"/>
-      <c r="H71" s="10" t="s">
+      <c r="F71" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G71" s="9"/>
+      <c r="H71" s="9" t="s">
         <v>61</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="14"/>
-      <c r="B72" s="14"/>
+      <c r="A72" s="16"/>
+      <c r="B72" s="16"/>
       <c r="C72" s="12"/>
       <c r="D72" s="13"/>
       <c r="E72" s="13"/>
       <c r="F72" s="13"/>
       <c r="G72" s="12"/>
-      <c r="H72" s="14"/>
-      <c r="I72" s="15"/>
+      <c r="H72" s="12"/>
+      <c r="I72" s="14"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B73" s="10"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="9"/>
-      <c r="F73" s="9"/>
-      <c r="G73" s="8"/>
-      <c r="H73" s="10"/>
-      <c r="I73" s="11"/>
+      <c r="A73" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C73" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D73" s="10"/>
+      <c r="E73" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F73" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H73" s="9"/>
+      <c r="I73" s="11" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B74" s="14"/>
+      <c r="A74" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="C74" s="12"/>
       <c r="D74" s="13"/>
-      <c r="E74" s="13"/>
+      <c r="E74" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="F74" s="13"/>
       <c r="G74" s="12"/>
-      <c r="H74" s="14"/>
-      <c r="I74" s="15"/>
+      <c r="H74" s="12"/>
+      <c r="I74" s="11" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B75" s="10"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="9"/>
-      <c r="E75" s="9"/>
-      <c r="F75" s="9"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="10"/>
-      <c r="I75" s="11"/>
+      <c r="A75" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C75" s="9"/>
+      <c r="D75" s="10"/>
+      <c r="E75" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F75" s="10"/>
+      <c r="G75" s="9"/>
+      <c r="H75" s="9"/>
+      <c r="I75" s="11" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B76" s="14"/>
+      <c r="A76" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>108</v>
+      </c>
       <c r="C76" s="12"/>
       <c r="D76" s="13"/>
-      <c r="E76" s="13"/>
+      <c r="E76" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="F76" s="13"/>
       <c r="G76" s="12"/>
-      <c r="H76" s="14"/>
-      <c r="I76" s="15"/>
+      <c r="H76" s="12"/>
+      <c r="I76" s="11" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B77" s="10"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="9"/>
-      <c r="F77" s="9"/>
-      <c r="G77" s="8"/>
-      <c r="H77" s="10"/>
-      <c r="I77" s="11"/>
+      <c r="A77" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C77" s="9"/>
+      <c r="D77" s="10"/>
+      <c r="E77" s="10"/>
+      <c r="F77" s="10"/>
+      <c r="G77" s="9"/>
+      <c r="H77" s="9"/>
+      <c r="I77" s="11" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B78" s="14"/>
+      <c r="A78" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>112</v>
+      </c>
       <c r="C78" s="12"/>
       <c r="D78" s="13"/>
       <c r="E78" s="13"/>
       <c r="F78" s="13"/>
       <c r="G78" s="12"/>
-      <c r="H78" s="14"/>
-      <c r="I78" s="15"/>
+      <c r="H78" s="12"/>
+      <c r="I78" s="11" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B79" s="10"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="9"/>
-      <c r="E79" s="9"/>
-      <c r="F79" s="9"/>
-      <c r="G79" s="8"/>
-      <c r="H79" s="10"/>
-      <c r="I79" s="11"/>
+      <c r="A79" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B79" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C79" s="9"/>
+      <c r="D79" s="10"/>
+      <c r="E79" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F79" s="10"/>
+      <c r="G79" s="9"/>
+      <c r="H79" s="9"/>
+      <c r="I79" s="11" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B80" s="14"/>
+      <c r="A80" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>116</v>
+      </c>
       <c r="C80" s="12"/>
       <c r="D80" s="13"/>
       <c r="E80" s="13"/>
       <c r="F80" s="13"/>
       <c r="G80" s="12"/>
-      <c r="H80" s="14"/>
-      <c r="I80" s="15"/>
+      <c r="H80" s="12"/>
+      <c r="I80" s="11" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B81" s="10"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="9"/>
-      <c r="E81" s="9"/>
-      <c r="F81" s="9"/>
-      <c r="G81" s="8"/>
-      <c r="H81" s="10"/>
-      <c r="I81" s="11"/>
+      <c r="A81" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B81" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C81" s="9"/>
+      <c r="D81" s="10"/>
+      <c r="E81" s="10"/>
+      <c r="F81" s="10"/>
+      <c r="G81" s="9"/>
+      <c r="H81" s="9"/>
+      <c r="I81" s="11" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B82" s="14"/>
+      <c r="A82" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>120</v>
+      </c>
       <c r="C82" s="12"/>
       <c r="D82" s="13"/>
       <c r="E82" s="13"/>
       <c r="F82" s="13"/>
       <c r="G82" s="12"/>
-      <c r="H82" s="14"/>
-      <c r="I82" s="15"/>
+      <c r="H82" s="12"/>
+      <c r="I82" s="14" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B83" s="10"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="9"/>
-      <c r="E83" s="9"/>
-      <c r="F83" s="9"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="10"/>
-      <c r="I83" s="11"/>
+      <c r="A83" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C83" s="9"/>
+      <c r="D83" s="10"/>
+      <c r="E83" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F83" s="10"/>
+      <c r="G83" s="9"/>
+      <c r="H83" s="9"/>
+      <c r="I83" s="11" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B84" s="14"/>
+      <c r="A84" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>124</v>
+      </c>
       <c r="C84" s="12"/>
       <c r="D84" s="13"/>
-      <c r="E84" s="13"/>
+      <c r="E84" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="F84" s="13"/>
       <c r="G84" s="12"/>
-      <c r="H84" s="14"/>
-      <c r="I84" s="15"/>
+      <c r="H84" s="12"/>
+      <c r="I84" s="14" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B85" s="10"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="9"/>
-      <c r="E85" s="9"/>
-      <c r="F85" s="9"/>
-      <c r="G85" s="8"/>
-      <c r="H85" s="10"/>
+      <c r="A85" s="17"/>
+      <c r="B85" s="17"/>
+      <c r="C85" s="9"/>
+      <c r="D85" s="10"/>
+      <c r="E85" s="10"/>
+      <c r="F85" s="10"/>
+      <c r="G85" s="9"/>
+      <c r="H85" s="9"/>
       <c r="I85" s="11"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B86" s="14"/>
+      <c r="A86" s="17"/>
+      <c r="B86" s="17"/>
       <c r="C86" s="12"/>
       <c r="D86" s="13"/>
       <c r="E86" s="13"/>
       <c r="F86" s="13"/>
       <c r="G86" s="12"/>
-      <c r="H86" s="14"/>
-      <c r="I86" s="15"/>
+      <c r="H86" s="12"/>
+      <c r="I86" s="14"/>
     </row>
     <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="10"/>
-      <c r="B87" s="10"/>
-      <c r="C87" s="8"/>
-      <c r="D87" s="9"/>
-      <c r="E87" s="9"/>
-      <c r="F87" s="9"/>
-      <c r="G87" s="8"/>
-      <c r="H87" s="10"/>
+      <c r="A87" s="15"/>
+      <c r="B87" s="15"/>
+      <c r="C87" s="9"/>
+      <c r="D87" s="10"/>
+      <c r="E87" s="10"/>
+      <c r="F87" s="10"/>
+      <c r="G87" s="9"/>
+      <c r="H87" s="9"/>
       <c r="I87" s="11"/>
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="14"/>
-      <c r="B88" s="14"/>
-      <c r="C88" s="12"/>
-      <c r="D88" s="13"/>
-      <c r="E88" s="13"/>
-      <c r="F88" s="13"/>
-      <c r="G88" s="12"/>
-      <c r="H88" s="14"/>
-      <c r="I88" s="15"/>
+      <c r="A88" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C88" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D88" s="10"/>
+      <c r="E88" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F88" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G88" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H88" s="9"/>
+      <c r="I88" s="11" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="10"/>
-      <c r="B89" s="10"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="9"/>
-      <c r="E89" s="9"/>
-      <c r="F89" s="9"/>
-      <c r="G89" s="8"/>
-      <c r="H89" s="10"/>
-      <c r="I89" s="11"/>
+      <c r="A89" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B89" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C89" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D89" s="10"/>
+      <c r="E89" s="10"/>
+      <c r="F89" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G89" s="9"/>
+      <c r="H89" s="9"/>
+      <c r="I89" s="11" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="14"/>
-      <c r="B90" s="14"/>
-      <c r="C90" s="12"/>
+      <c r="A90" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C90" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="D90" s="13"/>
       <c r="E90" s="13"/>
-      <c r="F90" s="13"/>
+      <c r="F90" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G90" s="12"/>
-      <c r="H90" s="14"/>
-      <c r="I90" s="15"/>
+      <c r="H90" s="12"/>
+      <c r="I90" s="14" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="10"/>
-      <c r="B91" s="10"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="9"/>
-      <c r="E91" s="9"/>
-      <c r="F91" s="9"/>
-      <c r="G91" s="8"/>
-      <c r="H91" s="10"/>
-      <c r="I91" s="11"/>
+      <c r="A91" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B91" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C91" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D91" s="10"/>
+      <c r="E91" s="10"/>
+      <c r="F91" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G91" s="9"/>
+      <c r="H91" s="9"/>
+      <c r="I91" s="11" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="14"/>
-      <c r="B92" s="14"/>
-      <c r="C92" s="12"/>
+      <c r="A92" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C92" s="12" t="s">
+        <v>136</v>
+      </c>
       <c r="D92" s="13"/>
       <c r="E92" s="13"/>
-      <c r="F92" s="13"/>
+      <c r="F92" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G92" s="12"/>
-      <c r="H92" s="14"/>
-      <c r="I92" s="15"/>
+      <c r="H92" s="12"/>
+      <c r="I92" s="14" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="10"/>
-      <c r="B93" s="10"/>
-      <c r="C93" s="8"/>
-      <c r="D93" s="9"/>
-      <c r="E93" s="9"/>
-      <c r="F93" s="9"/>
-      <c r="G93" s="8"/>
-      <c r="H93" s="10"/>
+      <c r="A93" s="17"/>
+      <c r="B93" s="17"/>
+      <c r="C93" s="9"/>
+      <c r="D93" s="10"/>
+      <c r="E93" s="10"/>
+      <c r="F93" s="10"/>
+      <c r="G93" s="9"/>
+      <c r="H93" s="9"/>
       <c r="I93" s="11"/>
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="14"/>
-      <c r="B94" s="14"/>
+      <c r="A94" s="17"/>
+      <c r="B94" s="17"/>
       <c r="C94" s="12"/>
       <c r="D94" s="13"/>
       <c r="E94" s="13"/>
       <c r="F94" s="13"/>
       <c r="G94" s="12"/>
-      <c r="H94" s="14"/>
-      <c r="I94" s="15"/>
+      <c r="H94" s="12"/>
+      <c r="I94" s="14"/>
     </row>
     <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="10"/>
-      <c r="B95" s="10"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="9"/>
-      <c r="E95" s="9"/>
-      <c r="F95" s="9"/>
-      <c r="G95" s="8"/>
-      <c r="H95" s="10"/>
+      <c r="A95" s="17"/>
+      <c r="B95" s="17"/>
+      <c r="C95" s="9"/>
+      <c r="D95" s="10"/>
+      <c r="E95" s="10"/>
+      <c r="F95" s="10"/>
+      <c r="G95" s="9"/>
+      <c r="H95" s="9"/>
       <c r="I95" s="11"/>
     </row>
-    <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A96" s="14"/>
-      <c r="B96" s="14"/>
-      <c r="C96" s="12"/>
-      <c r="D96" s="13"/>
-      <c r="E96" s="13"/>
-      <c r="F96" s="13"/>
-      <c r="G96" s="12"/>
-      <c r="H96" s="14"/>
-      <c r="I96" s="15"/>
-    </row>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B97" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="C97" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D97" s="10"/>
+      <c r="E97" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F97" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G97" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H97" s="9"/>
+      <c r="I97" s="11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B98" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I98" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B99" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I99" s="14" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B100" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I100" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B101" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="I101" s="14" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B102" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I102" s="14" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B103" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I103" s="14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B104" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I104" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B105" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I105" s="14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="19"/>
+      <c r="B106" s="19"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="19"/>
+      <c r="B107" s="19"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="19"/>
+      <c r="B108" s="19"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="19"/>
+      <c r="B109" s="19"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B110" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I110" s="14" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B111" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I111" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B112" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I112" s="14" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B113" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I113" s="14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B114" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I114" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B115" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I115" s="14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="19"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="19"/>
+    </row>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C96" type="list">
+  <dataValidations count="4">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C91 C93:C95 C97" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E96" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E95 E97" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F96" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F95 F97" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C92" type="list">
+      <formula1>Validações!$A$1:$A$12</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2685,133 +3228,133 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>95</v>
+      <c r="A1" s="3" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>96</v>
+      <c r="A2" s="4" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>98</v>
+      <c r="A4" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>100</v>
+      <c r="A5" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>102</v>
+      <c r="A6" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>104</v>
+      <c r="A7" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>106</v>
+      <c r="A8" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>108</v>
+      <c r="A9" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>110</v>
+      <c r="A10" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>112</v>
+      <c r="A11" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>114</v>
+      <c r="A12" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
-        <v>115</v>
+      <c r="A14" s="22" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="B16" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="I16" s="6" t="s">
+      <c r="G16" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>120</v>
+      <c r="A17" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>176</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>121</v>
+        <v>177</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>20</v>
@@ -2820,160 +3363,160 @@
         <v>21</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="H17" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>124</v>
+        <v>178</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>129</v>
+      <c r="A18" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="B19" s="14" t="s">
+      <c r="A19" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="B19" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>126</v>
+        <v>182</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>121</v>
+        <v>177</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>128</v>
+        <v>184</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="H19" s="14" t="s">
-        <v>130</v>
+        <v>179</v>
+      </c>
+      <c r="H19" s="16" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>133</v>
+      <c r="A20" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>134</v>
+      <c r="A21" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>190</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>126</v>
+        <v>182</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>127</v>
+        <v>183</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>128</v>
+        <v>184</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>40</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>136</v>
+        <v>191</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="E22" s="9" t="s">
+      <c r="A22" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="E22" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F22" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="H22" s="10" t="s">
-        <v>138</v>
+      <c r="F22" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>194</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>139</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>137</v>
+      <c r="A23" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>193</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>121</v>
+        <v>177</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>20</v>
@@ -2982,65 +3525,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="I23" s="15" t="s">
-        <v>141</v>
+        <v>178</v>
+      </c>
+      <c r="H23" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="H24" s="10" t="s">
-        <v>144</v>
+      <c r="A24" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>145</v>
+      <c r="A25" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>201</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>146</v>
+        <v>202</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>128</v>
+        <v>184</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>148</v>
+        <v>203</v>
+      </c>
+      <c r="H25" s="16" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -3059,7 +3602,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3075,7 +3618,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>149</v>
+        <v>205</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>28</v>
@@ -3086,23 +3629,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>150</v>
+        <v>206</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>151</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>152</v>
+        <v>208</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>128</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>153</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3112,27 +3655,32 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>154</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>132</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>155</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>156</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>157</v>
+        <v>213</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
criar tabela categoria servicos pecas
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="215">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -469,6 +469,9 @@
   </si>
   <si>
     <t xml:space="preserve">Campo da data de emissão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primária de identificação da categoria</t>
   </si>
   <si>
     <t xml:space="preserve">nome_categoria</t>
@@ -1168,14 +1171,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="33.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="45"/>
@@ -2982,6 +2986,9 @@
       <c r="C99" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="F99" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="I99" s="14" t="s">
         <v>144</v>
       </c>
@@ -3024,6 +3031,9 @@
       <c r="C102" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="F102" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="I102" s="14" t="s">
         <v>92</v>
       </c>
@@ -3038,6 +3048,9 @@
       <c r="C103" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="F103" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="I103" s="14" t="s">
         <v>93</v>
       </c>
@@ -3096,8 +3109,17 @@
       <c r="C110" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I110" s="14" t="s">
-        <v>144</v>
+      <c r="E110" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F110" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G110" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="I110" s="11" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3105,13 +3127,13 @@
         <v>131</v>
       </c>
       <c r="B111" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C111" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I111" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3124,6 +3146,9 @@
       <c r="C112" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="F112" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="I112" s="14" t="s">
         <v>92</v>
       </c>
@@ -3138,6 +3163,9 @@
       <c r="C113" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="F113" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="I113" s="14" t="s">
         <v>93</v>
       </c>
@@ -3176,21 +3204,17 @@
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="19"/>
     </row>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="4">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C91 C93:C95 C97" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E95 E97" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E95 E97 E110" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F95 F97" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F95 F97 F110" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3229,89 +3253,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3319,7 +3343,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>10</v>
@@ -3334,10 +3358,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>16</v>
@@ -3345,16 +3369,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>20</v>
@@ -3363,131 +3387,131 @@
         <v>21</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B19" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H19" s="16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>40</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>28</v>
@@ -3496,27 +3520,27 @@
         <v>21</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>20</v>
@@ -3525,65 +3549,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H23" s="16" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F24" s="10" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H25" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -3618,7 +3642,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>28</v>
@@ -3629,23 +3653,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3655,27 +3679,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>